<commit_message>
Re-run AMD COST NKE with latest engine
Score changes: COST +0.2, NKE -0.1, AMD -0.2
- COST: EM anchor 10x->21.2x, EM upside -48%->-28%
- NKE: EM anchor confirmed 19x, EM upside -13%->+35% (fresh data)
- AMD: forward P/E 65.7x scores LOW; EM upside -40%->-17% (28x cap)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/AMD_model.xlsx
+++ b/static/excel/AMD_model.xlsx
@@ -7358,11 +7358,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>733101.454</v>
+        <v>797681.367</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $449.59</t>
+          <t>FMP marketCap  |  price $489.195</t>
         </is>
       </c>
     </row>
@@ -7448,7 +7448,7 @@
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>FRED series DGS10  |  latest: 2026-05-20</t>
+          <t>FRED series DGS10  |  latest: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -7527,11 +7527,11 @@
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>Damodaran re-levered  (D/E = 0.01x,  t = 2.5%)</t>
+          <t>Damodaran re-levered  (D/E = 0.00x,  t = 2.5%)</t>
         </is>
       </c>
       <c r="B19" s="50" t="n">
-        <v>1.156</v>
+        <v>1.155</v>
       </c>
       <c r="C19" s="44">
         <f> unlevered × (1 + (1 − t) × D/E)</f>
@@ -7680,25 +7680,27 @@
       </c>
       <c r="B33" s="54" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>FMP /ratings endpoint</t>
+          <t>User input</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>FRED matched yield</t>
-        </is>
-      </c>
-      <c r="B34" s="54" t="n"/>
+          <t>FRED matched yield  (rating-tier index)</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="n">
+        <v>0.0507</v>
+      </c>
       <c r="C34" s="44" t="inlineStr">
         <is>
-          <t>No rating returned — FRED method not applicable</t>
+          <t>FRED BAMLC0A3CAEY — A</t>
         </is>
       </c>
     </row>
@@ -7784,11 +7786,11 @@
         </is>
       </c>
       <c r="B40" s="48" t="n">
-        <v>0.0491</v>
+        <v>0.0496</v>
       </c>
       <c r="C40" s="49" t="inlineStr">
         <is>
-          <t>Default = average of 2 source(s) above — override freely</t>
+          <t>Default = average of 3 source(s) above — override freely</t>
         </is>
       </c>
     </row>
@@ -7849,16 +7851,16 @@
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="55" t="inlineStr">
         <is>
-          <t>WACC  =  (E/V × Re)  +  (D/V × Rd × (1 − t))</t>
+          <t>WACC  =  MAX(8.5%, (E/V × Re) + (D/V × Rd × (1 − t)))</t>
         </is>
       </c>
       <c r="B47" s="56">
-        <f>B8*B30+B9*B40*(1-B44)</f>
+        <f>MAX(0.085, B8*B30+B9*B40*(1-B44))</f>
         <v/>
       </c>
       <c r="C47" s="57" t="inlineStr">
         <is>
-          <t>Used as discount rate in DCF tab</t>
+          <t>Floored 8.5% (D-001); raw formula below</t>
         </is>
       </c>
     </row>
@@ -8222,13 +8224,13 @@
         <v/>
       </c>
       <c r="G7" s="72" t="n">
-        <v>0.4343</v>
+        <v>0.4396</v>
       </c>
       <c r="H7" s="72" t="n">
-        <v>0.5263</v>
+        <v>0.5296999999999999</v>
       </c>
       <c r="I7" s="72" t="n">
-        <v>0.3242</v>
+        <v>0.326</v>
       </c>
       <c r="J7" s="73">
         <f>I7</f>
@@ -8572,13 +8574,13 @@
         <v/>
       </c>
       <c r="G15" s="78" t="n">
-        <v>49684.3</v>
+        <v>49865.9</v>
       </c>
       <c r="H15" s="78" t="n">
-        <v>75831.89999999999</v>
+        <v>76280.2</v>
       </c>
       <c r="I15" s="78" t="n">
-        <v>100413.1</v>
+        <v>101145.4</v>
       </c>
       <c r="J15" s="79">
         <f>I15*(1+J7)</f>
@@ -8606,27 +8608,27 @@
       </c>
       <c r="G16" s="83" t="inlineStr">
         <is>
-          <t>42,464 — 51,623</t>
+          <t>42,619 — 51,812</t>
         </is>
       </c>
       <c r="H16" s="83" t="inlineStr">
         <is>
-          <t>56,415 — 83,223</t>
+          <t>56,749 — 83,715</t>
         </is>
       </c>
       <c r="I16" s="83" t="inlineStr">
         <is>
-          <t>100,345 — 100,481</t>
+          <t>100,368 — 101,923</t>
         </is>
       </c>
       <c r="J16" s="83" t="inlineStr">
         <is>
-          <t>117,074 — 167,118</t>
+          <t>116,659 — 168,232</t>
         </is>
       </c>
       <c r="K16" s="83" t="inlineStr">
         <is>
-          <t>139,069 — 198,515</t>
+          <t>138,576 — 199,838</t>
         </is>
       </c>
       <c r="L16" s="84" t="inlineStr">
@@ -8647,19 +8649,19 @@
         </is>
       </c>
       <c r="G17" s="85" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H17" s="85" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I17" s="85" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J17" s="85" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="K17" s="85" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="L17" s="84" t="inlineStr">
         <is>
@@ -8770,13 +8772,13 @@
         <v/>
       </c>
       <c r="G20" s="78" t="n">
-        <v>10780.1</v>
+        <v>10819.5</v>
       </c>
       <c r="H20" s="78" t="n">
-        <v>16453.4</v>
+        <v>16550.6</v>
       </c>
       <c r="I20" s="78" t="n">
-        <v>21786.8</v>
+        <v>21945.7</v>
       </c>
       <c r="J20" s="79">
         <f>J15*J8</f>
@@ -8804,27 +8806,27 @@
       </c>
       <c r="G21" s="83" t="inlineStr">
         <is>
-          <t>9,214 — 11,201</t>
+          <t>9,247 — 11,242</t>
         </is>
       </c>
       <c r="H21" s="83" t="inlineStr">
         <is>
-          <t>12,241 — 18,057</t>
+          <t>12,313 — 18,164</t>
         </is>
       </c>
       <c r="I21" s="83" t="inlineStr">
         <is>
-          <t>21,772 — 21,801</t>
+          <t>21,777 — 22,114</t>
         </is>
       </c>
       <c r="J21" s="83" t="inlineStr">
         <is>
-          <t>25,402 — 36,260</t>
+          <t>25,312 — 36,501</t>
         </is>
       </c>
       <c r="K21" s="83" t="inlineStr">
         <is>
-          <t>30,174 — 43,072</t>
+          <t>30,067 — 43,359</t>
         </is>
       </c>
       <c r="L21" s="84" t="inlineStr">
@@ -9488,7 +9490,7 @@
         </is>
       </c>
       <c r="B38" s="101" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C38" s="99" t="n"/>
       <c r="D38" s="99" t="n"/>
@@ -9502,7 +9504,7 @@
       <c r="L38" s="99" t="n"/>
       <c r="M38" s="75" t="inlineStr">
         <is>
-          <t>Growth tier: HIGH (14.7% 3yr avg rev growth).  Bear 14x / Base 18x / Bull 22x.  Override manually if needed.</t>
+          <t>Growth tier: HIGH (14.7% 3yr avg rev growth).  Bear 22x / Base 28x / Bull 32x.  Override manually if needed.</t>
         </is>
       </c>
     </row>
@@ -10004,7 +10006,7 @@
         </is>
       </c>
       <c r="B61" s="112" t="n">
-        <v>449.59</v>
+        <v>489.19</v>
       </c>
       <c r="C61" s="104" t="n"/>
       <c r="D61" s="104" t="n"/>
@@ -10104,7 +10106,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="114" t="inlineStr">
         <is>
-          <t>JS SCORECARD — AMD  |  Master Prompt v2  |  22 May 2026  |  Sector bucket: Tech Growth</t>
+          <t>JS SCORECARD — AMD  |  Master Prompt v2  |  26 May 2026  |  Sector bucket: Tech Growth</t>
         </is>
       </c>
     </row>
@@ -10621,7 +10623,7 @@
       </c>
       <c r="D22" s="130" t="inlineStr">
         <is>
-          <t>Current 80.5x  |  5yr avg 123.1x  |  Sector median 28.5x  |  DCF-implied 59.6x [ref only — not used as benchmark]  [+182% vs benchmark]  [trail=0.00 | no_fwd_data(fallback) | abs=0.0 → blended 40/40/20=0.00]  PEG≈590.02 (trailing_pe=80.5x / rev_cagr=14%, revenue proxy)</t>
+          <t>Fwd P/E 65.7x (scoring basis)  |  5yr avg 123.1x  |  Sector median 28.5x  |  DCF-implied 60.2x [ref only — not used as benchmark]  [+131% vs benchmark]  [trail=0.00 | fwd_pe=65.7x→0.00 | abs=0.0 → blended 40/40/20=0.00]  PEG=36.74 (fwd_pe=65.7x / eps_growth=179%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
       <c r="E22" s="136" t="inlineStr">
@@ -10630,7 +10632,7 @@
         </is>
       </c>
       <c r="F22" s="132" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G22" s="133">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10638,7 +10640,7 @@
       </c>
       <c r="H22" s="134" t="inlineStr">
         <is>
-          <t>Current 80.5x  |  5yr avg 123.1x  |  Sector median 28.5x  |  DCF-implied 59.6x [ref only — not used as benchmark]  [+182% vs benchmark]  [trail=0.00 | no_fwd_data(fallback) | abs=0.0 → blended 40/40/20=0.00]  PEG≈590.02 (trailing_pe=80.5x / rev_cagr=14%, revenue proxy)</t>
+          <t>Fwd P/E 65.7x (scoring basis)  |  5yr avg 123.1x  |  Sector median 28.5x  |  DCF-implied 60.2x [ref only — not used as benchmark]  [+131% vs benchmark]  [trail=0.00 | fwd_pe=65.7x→0.00 | abs=0.0 → blended 40/40/20=0.00]  PEG=36.74 (fwd_pe=65.7x / eps_growth=179%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
     </row>
@@ -10658,7 +10660,7 @@
       </c>
       <c r="D23" s="130" t="inlineStr">
         <is>
-          <t>Current 51.8x  |  5yr avg 87.2x  |  Sector median 45.0x  |  DCF-implied 38.4x [ref only — not used as benchmark]  [+15% vs benchmark]  [trail=4.58 | no_fwd_data(fallback) | abs=1.5 → blended 40/40/20=3.97]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
+          <t>Current 51.8x  |  5yr avg 87.2x  |  Sector median 45.0x  |  DCF-implied 38.7x [ref only — not used as benchmark]  [+15% vs benchmark]  [trail=4.58 | fwd_pfcf=81.9x→0.00 | abs=1.5 → blended 40/40/20=2.13]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
         </is>
       </c>
       <c r="E23" s="131" t="inlineStr">
@@ -10667,7 +10669,7 @@
         </is>
       </c>
       <c r="F23" s="132" t="n">
-        <v>3.47</v>
+        <v>1.63</v>
       </c>
       <c r="G23" s="133">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10675,7 +10677,7 @@
       </c>
       <c r="H23" s="134" t="inlineStr">
         <is>
-          <t>Current 51.8x  |  5yr avg 87.2x  |  Sector median 45.0x  |  DCF-implied 38.4x [ref only — not used as benchmark]  [+15% vs benchmark]  [trail=4.58 | no_fwd_data(fallback) | abs=1.5 → blended 40/40/20=3.97]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
+          <t>Current 51.8x  |  5yr avg 87.2x  |  Sector median 45.0x  |  DCF-implied 38.7x [ref only — not used as benchmark]  [+15% vs benchmark]  [trail=4.58 | fwd_pfcf=81.9x→0.00 | abs=1.5 → blended 40/40/20=2.13]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
         </is>
       </c>
     </row>

</xml_diff>